<commit_message>
ci: regenera página y Excel
</commit_message>
<xml_diff>
--- a/docs/research.xlsx
+++ b/docs/research.xlsx
@@ -21319,7 +21319,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Reino Unido</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -21461,7 +21461,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Reino Unido</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -22258,7 +22258,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -22381,7 +22381,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -23846,7 +23846,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Espana</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -23967,7 +23967,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Espana</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -24209,7 +24209,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Reino Unido</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -24330,7 +24330,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Espana</t>
+          <t>Spain</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">

</xml_diff>